<commit_message>
Welcome TrueHold Wellness customers with the official logo and decrement inventory on orders.
/start now sends logo.jpeg plus a short how-it-works intro. Confirmed interest orders adjust on-hand stock and the orders workbook the same way as the old ledger.

Co-authored-by: James Rupe <cardanomint@gmail.com>
</commit_message>
<xml_diff>
--- a/truehold-wellness/wellness_agent/inventory/workbooks/trueholdwellness-orders.xlsx
+++ b/truehold-wellness/wellness_agent/inventory/workbooks/trueholdwellness-orders.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Clients" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inventory'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inventory'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Orders'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Payments'!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Fulfillment'!$A$1:$F$1</definedName>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="88" customWidth="1" min="1" max="1"/>
@@ -550,6 +550,30 @@
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>The team calls to confirm, consult, and complete required documentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Fill Inventory.on_hand with live vial counts, then ingest-files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Telegram interest orders decrement on-hand the same way as before.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Leave on_hand blank until you have a real count — do not invent stock.</t>
         </is>
       </c>
     </row>
@@ -564,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -575,6 +599,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -618,6 +643,11 @@
           <t>fulfillment</t>
         </is>
       </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>on_hand</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -660,6 +690,7 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -702,6 +733,7 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -744,6 +776,7 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -786,6 +819,7 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -828,6 +862,7 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -870,6 +905,7 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -912,6 +948,7 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -954,9 +991,10 @@
           <t>Las Vegas prep/delivery; dry-vial ship only</t>
         </is>
       </c>
+      <c r="I9" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>